<commit_message>
Expanded passenger dataset to 30 observations
Added 22 new passenger observations, increasing the dataset from 8 to 30
</commit_message>
<xml_diff>
--- a/100 Passengers Data Project.xlsx
+++ b/100 Passengers Data Project.xlsx
@@ -1,21 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11023"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://cityuni-my.sharepoint.com/personal/jeremy_nwosu_city_ac_uk/Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{9CAC6715-9069-4EDA-AD2B-9B32A0B8CE99}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="127" documentId="8_{9CAC6715-9069-4EDA-AD2B-9B32A0B8CE99}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E2314EF7-ABA9-174C-A435-F46AFD96B193}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{EA8149E3-4800-440C-85A1-B8CA984A9C47}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="191028"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="150" uniqueCount="34">
   <si>
     <t>Train Type</t>
   </si>
@@ -102,6 +102,45 @@
   </si>
   <si>
     <t>Back</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sitting </t>
+  </si>
+  <si>
+    <t>Seat</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Wireless Headphones </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Wired Headphones </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Listening </t>
+  </si>
+  <si>
+    <t>Newspaper</t>
+  </si>
+  <si>
+    <t>Wireless Earphones</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Standing </t>
+  </si>
+  <si>
+    <t>Shoulder</t>
+  </si>
+  <si>
+    <t xml:space="preserve">None </t>
+  </si>
+  <si>
+    <t>Talking</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Underground </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Wired Earphones </t>
   </si>
 </sst>
 </file>
@@ -510,18 +549,18 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{89EDB40A-A8F8-45B7-8805-F02DF0852829}">
-  <dimension ref="A1:E8"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:E30"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="16.5703125" customWidth="1"/>
-    <col min="2" max="2" width="20.28515625" customWidth="1"/>
-    <col min="3" max="3" width="9.85546875" customWidth="1"/>
-    <col min="4" max="4" width="20" customWidth="1"/>
+    <col min="1" max="1" width="16.54296875" customWidth="1"/>
+    <col min="2" max="2" width="20.3125" customWidth="1"/>
+    <col min="3" max="3" width="9.81640625" customWidth="1"/>
+    <col min="4" max="4" width="20.04296875" customWidth="1"/>
     <col min="5" max="5" width="13.85546875" customWidth="1"/>
-    <col min="6" max="6" width="11" customWidth="1"/>
+    <col min="6" max="6" width="11.02734375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -538,7 +577,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A2" s="2" t="s">
         <v>6</v>
       </c>
@@ -555,7 +594,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>6</v>
       </c>
@@ -572,7 +611,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>7</v>
       </c>
@@ -589,7 +628,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>6</v>
       </c>
@@ -606,7 +645,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>7</v>
       </c>
@@ -623,7 +662,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>7</v>
       </c>
@@ -640,7 +679,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>6</v>
       </c>
@@ -655,6 +694,380 @@
       </c>
       <c r="E8" t="s">
         <v>15</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A9" t="s">
+        <v>7</v>
+      </c>
+      <c r="B9" t="s">
+        <v>21</v>
+      </c>
+      <c r="C9" t="s">
+        <v>13</v>
+      </c>
+      <c r="D9" t="s">
+        <v>10</v>
+      </c>
+      <c r="E9" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A10" t="s">
+        <v>7</v>
+      </c>
+      <c r="B10" t="s">
+        <v>12</v>
+      </c>
+      <c r="C10" t="s">
+        <v>16</v>
+      </c>
+      <c r="D10" t="s">
+        <v>23</v>
+      </c>
+      <c r="E10" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A11" t="s">
+        <v>7</v>
+      </c>
+      <c r="B11" t="s">
+        <v>12</v>
+      </c>
+      <c r="C11" t="s">
+        <v>16</v>
+      </c>
+      <c r="D11" t="s">
+        <v>14</v>
+      </c>
+      <c r="E11" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A12" t="s">
+        <v>7</v>
+      </c>
+      <c r="B12" t="s">
+        <v>12</v>
+      </c>
+      <c r="C12" t="s">
+        <v>16</v>
+      </c>
+      <c r="D12" t="s">
+        <v>24</v>
+      </c>
+      <c r="E12" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A13" t="s">
+        <v>7</v>
+      </c>
+      <c r="B13" t="s">
+        <v>12</v>
+      </c>
+      <c r="C13" t="s">
+        <v>25</v>
+      </c>
+      <c r="D13" t="s">
+        <v>14</v>
+      </c>
+      <c r="E13" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A14" t="s">
+        <v>6</v>
+      </c>
+      <c r="B14" t="s">
+        <v>12</v>
+      </c>
+      <c r="C14" t="s">
+        <v>26</v>
+      </c>
+      <c r="D14" t="s">
+        <v>10</v>
+      </c>
+      <c r="E14" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A15" t="s">
+        <v>6</v>
+      </c>
+      <c r="B15" t="s">
+        <v>12</v>
+      </c>
+      <c r="C15" t="s">
+        <v>18</v>
+      </c>
+      <c r="D15" t="s">
+        <v>27</v>
+      </c>
+      <c r="E15" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A16" t="s">
+        <v>6</v>
+      </c>
+      <c r="B16" t="s">
+        <v>28</v>
+      </c>
+      <c r="C16" t="s">
+        <v>25</v>
+      </c>
+      <c r="D16" t="s">
+        <v>23</v>
+      </c>
+      <c r="E16" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A17" t="s">
+        <v>6</v>
+      </c>
+      <c r="B17" t="s">
+        <v>8</v>
+      </c>
+      <c r="C17" t="s">
+        <v>16</v>
+      </c>
+      <c r="D17" t="s">
+        <v>27</v>
+      </c>
+      <c r="E17" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A18" t="s">
+        <v>6</v>
+      </c>
+      <c r="B18" t="s">
+        <v>8</v>
+      </c>
+      <c r="C18" t="s">
+        <v>18</v>
+      </c>
+      <c r="D18" t="s">
+        <v>14</v>
+      </c>
+      <c r="E18" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A19" t="s">
+        <v>6</v>
+      </c>
+      <c r="B19" t="s">
+        <v>28</v>
+      </c>
+      <c r="C19" t="s">
+        <v>10</v>
+      </c>
+      <c r="D19" t="s">
+        <v>30</v>
+      </c>
+      <c r="E19" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A20" t="s">
+        <v>7</v>
+      </c>
+      <c r="B20" t="s">
+        <v>28</v>
+      </c>
+      <c r="C20" t="s">
+        <v>16</v>
+      </c>
+      <c r="D20" t="s">
+        <v>30</v>
+      </c>
+      <c r="E20" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A21" t="s">
+        <v>6</v>
+      </c>
+      <c r="B21" t="s">
+        <v>8</v>
+      </c>
+      <c r="C21" t="s">
+        <v>9</v>
+      </c>
+      <c r="D21" t="s">
+        <v>10</v>
+      </c>
+      <c r="E21" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A22" t="s">
+        <v>6</v>
+      </c>
+      <c r="B22" t="s">
+        <v>8</v>
+      </c>
+      <c r="C22" t="s">
+        <v>31</v>
+      </c>
+      <c r="D22" t="s">
+        <v>10</v>
+      </c>
+      <c r="E22" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A23" t="s">
+        <v>6</v>
+      </c>
+      <c r="B23" t="s">
+        <v>8</v>
+      </c>
+      <c r="C23" t="s">
+        <v>31</v>
+      </c>
+      <c r="D23" t="s">
+        <v>10</v>
+      </c>
+      <c r="E23" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A24" t="s">
+        <v>6</v>
+      </c>
+      <c r="B24" t="s">
+        <v>12</v>
+      </c>
+      <c r="C24" t="s">
+        <v>9</v>
+      </c>
+      <c r="D24" t="s">
+        <v>10</v>
+      </c>
+      <c r="E24" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A25" t="s">
+        <v>6</v>
+      </c>
+      <c r="B25" t="s">
+        <v>12</v>
+      </c>
+      <c r="C25" t="s">
+        <v>18</v>
+      </c>
+      <c r="D25" t="s">
+        <v>19</v>
+      </c>
+      <c r="E25" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A26" t="s">
+        <v>6</v>
+      </c>
+      <c r="B26" t="s">
+        <v>21</v>
+      </c>
+      <c r="C26" t="s">
+        <v>16</v>
+      </c>
+      <c r="D26" t="s">
+        <v>27</v>
+      </c>
+      <c r="E26" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A27" t="s">
+        <v>6</v>
+      </c>
+      <c r="B27" t="s">
+        <v>12</v>
+      </c>
+      <c r="C27" t="s">
+        <v>16</v>
+      </c>
+      <c r="D27" t="s">
+        <v>27</v>
+      </c>
+      <c r="E27" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A28" t="s">
+        <v>32</v>
+      </c>
+      <c r="B28" t="s">
+        <v>21</v>
+      </c>
+      <c r="C28" t="s">
+        <v>16</v>
+      </c>
+      <c r="D28" t="s">
+        <v>33</v>
+      </c>
+      <c r="E28" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A29" t="s">
+        <v>7</v>
+      </c>
+      <c r="B29" t="s">
+        <v>21</v>
+      </c>
+      <c r="C29" t="s">
+        <v>31</v>
+      </c>
+      <c r="D29" t="s">
+        <v>27</v>
+      </c>
+      <c r="E29" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A30" t="s">
+        <v>7</v>
+      </c>
+      <c r="B30" t="s">
+        <v>21</v>
+      </c>
+      <c r="C30" t="s">
+        <v>16</v>
+      </c>
+      <c r="D30" t="s">
+        <v>19</v>
+      </c>
+      <c r="E30" t="s">
+        <v>11</v>
       </c>
     </row>
   </sheetData>
@@ -836,6 +1249,12 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
   <Display>DocumentLibraryForm</Display>
@@ -844,50 +1263,31 @@
 </FormTemplates>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3F6CD6A1-EC4E-4A84-B5FC-CF531BE122F9}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2000/xmlns/"/>
     <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
     <ds:schemaRef ds:uri="75eb23ce-bee3-4614-ac9d-e7493ba98713"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{939CEE1B-FD12-4D29-A50D-9ED00F07F23D}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2000/xmlns/"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{73173EA6-72A4-4717-ADEE-037D49EB9844}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{939CEE1B-FD12-4D29-A50D-9ED00F07F23D}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="75eb23ce-bee3-4614-ac9d-e7493ba98713"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>